<commit_message>
Add lesson room constraints and localize class preferences
</commit_message>
<xml_diff>
--- a/Testy/NauczycieleSP3Bielawa.xlsx
+++ b/Testy/NauczycieleSP3Bielawa.xlsx
@@ -13,7 +13,7 @@
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1"/>
+      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -173,7 +173,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -194,13 +194,49 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF81D41A"/>
+        <bgColor rgb="FFE6E905"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB66C"/>
+        <bgColor rgb="FFFF99CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB4C7DC"/>
+        <bgColor rgb="FFCCCCFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF800080"/>
+        <bgColor rgb="FF800080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6E905"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -237,8 +273,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -251,6 +307,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFE6E905"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFB4C7DC"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFB66C"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF81D41A"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -372,75 +488,75 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.33"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -468,35 +584,35 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+    <row r="13" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+    <row r="14" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+    <row r="16" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="3" t="s">
         <v>20</v>
       </c>
     </row>
@@ -564,35 +680,35 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+    <row r="25" s="4" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+    <row r="26" s="5" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+    <row r="27" s="5" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+    <row r="28" s="5" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="5" t="s">
         <v>43</v>
       </c>
     </row>
@@ -614,11 +730,11 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regularna"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regularna"&amp;12Strona &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;CStrona &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>